<commit_message>
Add some new files
</commit_message>
<xml_diff>
--- a/2025年迎新杯/义工活动/志愿者名单及时长统计/南科大义工联志愿服务活动签到、签退表.xlsx
+++ b/2025年迎新杯/义工活动/志愿者名单及时长统计/南科大义工联志愿服务活动签到、签退表.xlsx
@@ -5,17 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kaichengmao/Documents/排球社2025-2026学年/2025年迎新杯/义工活动/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kaichengmao/Documents/排球社2025-2026学年/2025年迎新杯/义工活动/志愿者名单及时长统计/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E277B0D-1986-2944-8E97-F54FAE1FA194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A8355A2-0324-0940-9D6F-F143685DB50E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="16000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$O$1:$T$32</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -32,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="259">
   <si>
     <t>南科大义工队志愿服务活动签到、签退表</t>
   </si>
@@ -902,6 +905,9 @@
   <si>
     <t>97</t>
     <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <t>27</t>
   </si>
 </sst>
 </file>
@@ -1054,7 +1060,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1130,44 +1136,47 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2965,6 +2974,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB163"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="18"/>
   <cols>
@@ -2991,25 +3003,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="1" customFormat="1" ht="45" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
       <c r="L1" s="22"/>
-      <c r="O1" s="32" t="s">
+      <c r="O1" s="38" t="s">
         <v>191</v>
       </c>
-      <c r="P1" s="33"/>
-      <c r="Q1" s="33"/>
-      <c r="R1" s="33"/>
-      <c r="S1" s="33"/>
-      <c r="T1" s="34"/>
+      <c r="P1" s="39"/>
+      <c r="Q1" s="39"/>
+      <c r="R1" s="39"/>
+      <c r="S1" s="39"/>
+      <c r="T1" s="40"/>
     </row>
     <row r="2" spans="1:28" s="2" customFormat="1" ht="36" customHeight="1">
       <c r="A2" s="7"/>
@@ -3044,22 +3056,22 @@
       <c r="L2" s="23"/>
       <c r="M2" s="13"/>
       <c r="N2" s="13"/>
-      <c r="O2" s="2" t="s">
+      <c r="O2" s="31" t="s">
         <v>192</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="P2" s="31" t="s">
         <v>193</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="Q2" s="31" t="s">
         <v>194</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="R2" s="31" t="s">
         <v>252</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="S2" s="31" t="s">
         <v>195</v>
       </c>
-      <c r="T2" s="2" t="s">
+      <c r="T2" s="31" t="s">
         <v>196</v>
       </c>
     </row>
@@ -3094,20 +3106,20 @@
       <c r="L3" s="16"/>
       <c r="M3" s="15"/>
       <c r="N3" s="16"/>
-      <c r="O3" s="27">
+      <c r="O3" s="17">
         <v>1</v>
       </c>
-      <c r="P3" s="28" t="s">
+      <c r="P3" s="27" t="s">
         <v>197</v>
       </c>
-      <c r="Q3" s="31" t="s">
+      <c r="Q3" s="32" t="s">
         <v>198</v>
       </c>
-      <c r="R3" s="27">
+      <c r="R3" s="17">
         <f ca="1">SUMIF(C3:C98,Q3,H3:H94)</f>
         <v>10.5</v>
       </c>
-      <c r="S3" s="27" t="s">
+      <c r="S3" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T3" s="9" t="s">
@@ -3150,20 +3162,20 @@
       <c r="L4" s="16"/>
       <c r="M4" s="15"/>
       <c r="N4" s="16"/>
-      <c r="O4" s="3">
+      <c r="O4" s="33">
         <v>2</v>
       </c>
-      <c r="P4" s="29" t="s">
+      <c r="P4" s="27" t="s">
         <v>199</v>
       </c>
-      <c r="Q4" s="31" t="s">
+      <c r="Q4" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="R4" s="27">
+      <c r="R4" s="17">
         <f ca="1">SUMIF(C3:C98,Q4,H3:H94)</f>
         <v>16.5</v>
       </c>
-      <c r="S4" s="27" t="s">
+      <c r="S4" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T4" s="9" t="s">
@@ -3207,20 +3219,20 @@
       <c r="L5" s="16"/>
       <c r="M5" s="15"/>
       <c r="N5" s="16"/>
-      <c r="O5" s="27">
+      <c r="O5" s="17">
         <v>3</v>
       </c>
-      <c r="P5" s="28" t="s">
+      <c r="P5" s="27" t="s">
         <v>200</v>
       </c>
-      <c r="Q5" s="31" t="s">
+      <c r="Q5" s="32" t="s">
         <v>225</v>
       </c>
-      <c r="R5" s="27">
+      <c r="R5" s="17">
         <f ca="1">SUMIF(C3:C98,Q5,H3:H94)</f>
         <v>7.5</v>
       </c>
-      <c r="S5" s="27" t="s">
+      <c r="S5" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T5" s="9" t="s">
@@ -3258,20 +3270,20 @@
       <c r="L6" s="16"/>
       <c r="M6" s="15"/>
       <c r="N6" s="16"/>
-      <c r="O6" s="27">
+      <c r="O6" s="17">
         <v>4</v>
       </c>
-      <c r="P6" s="28" t="s">
+      <c r="P6" s="27" t="s">
         <v>201</v>
       </c>
-      <c r="Q6" s="31" t="s">
+      <c r="Q6" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="R6" s="27">
+      <c r="R6" s="17">
         <f ca="1">SUMIF(C3:C98,Q6,H3:H94)</f>
         <v>7.5</v>
       </c>
-      <c r="S6" s="27" t="s">
+      <c r="S6" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T6" s="9" t="s">
@@ -3309,20 +3321,20 @@
       <c r="L7" s="15"/>
       <c r="M7" s="15"/>
       <c r="N7" s="16"/>
-      <c r="O7" s="27">
+      <c r="O7" s="17">
         <v>5</v>
       </c>
-      <c r="P7" s="28" t="s">
+      <c r="P7" s="27" t="s">
         <v>202</v>
       </c>
-      <c r="Q7" s="31" t="s">
+      <c r="Q7" s="32" t="s">
         <v>148</v>
       </c>
-      <c r="R7" s="27">
+      <c r="R7" s="17">
         <f ca="1">SUMIF(C3:C98,Q7,H3:H94)</f>
         <v>1.5</v>
       </c>
-      <c r="S7" s="27" t="s">
+      <c r="S7" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T7" s="9" t="s">
@@ -3360,20 +3372,20 @@
       <c r="L8" s="16"/>
       <c r="M8" s="15"/>
       <c r="N8" s="16"/>
-      <c r="O8" s="27">
+      <c r="O8" s="17">
         <v>6</v>
       </c>
-      <c r="P8" s="28" t="s">
+      <c r="P8" s="27" t="s">
         <v>203</v>
       </c>
-      <c r="Q8" s="31" t="s">
+      <c r="Q8" s="32" t="s">
         <v>226</v>
       </c>
-      <c r="R8" s="27">
+      <c r="R8" s="17">
         <f>SUMIF(C3:C94,Q8,H3:H94)</f>
         <v>0</v>
       </c>
-      <c r="S8" s="27" t="s">
+      <c r="S8" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T8" s="9" t="s">
@@ -3411,20 +3423,20 @@
       <c r="L9" s="16"/>
       <c r="M9" s="15"/>
       <c r="N9" s="16"/>
-      <c r="O9" s="27">
+      <c r="O9" s="17">
         <v>7</v>
       </c>
-      <c r="P9" s="28" t="s">
+      <c r="P9" s="27" t="s">
         <v>204</v>
       </c>
-      <c r="Q9" s="31" t="s">
+      <c r="Q9" s="32" t="s">
         <v>227</v>
       </c>
-      <c r="R9" s="27">
+      <c r="R9" s="17">
         <f>SUMIF(C3:C98,Q9,H3:H100)</f>
         <v>4.5</v>
       </c>
-      <c r="S9" s="27" t="s">
+      <c r="S9" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T9" s="9" t="s">
@@ -3462,20 +3474,20 @@
       <c r="L10" s="16"/>
       <c r="M10" s="15"/>
       <c r="N10" s="16"/>
-      <c r="O10" s="27">
+      <c r="O10" s="17">
         <v>8</v>
       </c>
-      <c r="P10" s="28" t="s">
+      <c r="P10" s="27" t="s">
         <v>205</v>
       </c>
-      <c r="Q10" s="31" t="s">
+      <c r="Q10" s="32" t="s">
         <v>228</v>
       </c>
-      <c r="R10" s="27">
+      <c r="R10" s="17">
         <f>SUMIF(C3:C100,Q10,H3:H100)</f>
         <v>3</v>
       </c>
-      <c r="S10" s="27" t="s">
+      <c r="S10" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T10" s="9" t="s">
@@ -3513,20 +3525,20 @@
       <c r="L11" s="16"/>
       <c r="M11" s="15"/>
       <c r="N11" s="16"/>
-      <c r="O11" s="27">
+      <c r="O11" s="17">
         <v>9</v>
       </c>
-      <c r="P11" s="28" t="s">
+      <c r="P11" s="27" t="s">
         <v>206</v>
       </c>
-      <c r="Q11" s="31" t="s">
+      <c r="Q11" s="32" t="s">
         <v>229</v>
       </c>
-      <c r="R11" s="27">
+      <c r="R11" s="17">
         <f>SUMIF(C3:C100,Q11,H3:H100)</f>
         <v>10.5</v>
       </c>
-      <c r="S11" s="27" t="s">
+      <c r="S11" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T11" s="9" t="s">
@@ -3564,20 +3576,20 @@
       <c r="L12" s="16"/>
       <c r="M12" s="15"/>
       <c r="N12" s="16"/>
-      <c r="O12" s="27">
+      <c r="O12" s="17">
         <v>10</v>
       </c>
-      <c r="P12" s="30" t="s">
+      <c r="P12" s="28" t="s">
         <v>207</v>
       </c>
-      <c r="Q12" s="37" t="s">
+      <c r="Q12" s="34" t="s">
         <v>248</v>
       </c>
-      <c r="R12" s="27">
+      <c r="R12" s="17">
         <f>SUMIF(C3:C100,Q12,H3:H100)</f>
         <v>7.5</v>
       </c>
-      <c r="S12" s="27" t="s">
+      <c r="S12" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T12" s="9" t="s">
@@ -3615,20 +3627,20 @@
       <c r="L13" s="16"/>
       <c r="M13" s="15"/>
       <c r="N13" s="16"/>
-      <c r="O13" s="27">
+      <c r="O13" s="17">
         <v>11</v>
       </c>
-      <c r="P13" s="29" t="s">
+      <c r="P13" s="27" t="s">
         <v>208</v>
       </c>
-      <c r="Q13" s="31" t="s">
+      <c r="Q13" s="32" t="s">
         <v>230</v>
       </c>
-      <c r="R13" s="27">
+      <c r="R13" s="17">
         <f>SUMIF(C3:C105,Q13,H3:H105)</f>
         <v>12</v>
       </c>
-      <c r="S13" s="27" t="s">
+      <c r="S13" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T13" s="9" t="s">
@@ -3662,20 +3674,20 @@
       <c r="J14" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="O14" s="3">
+      <c r="O14" s="33">
         <v>12</v>
       </c>
-      <c r="P14" s="29" t="s">
+      <c r="P14" s="27" t="s">
         <v>209</v>
       </c>
-      <c r="Q14" s="31" t="s">
+      <c r="Q14" s="32" t="s">
         <v>231</v>
       </c>
-      <c r="R14" s="27">
+      <c r="R14" s="17">
         <f>SUMIF(C33:C105,Q14,H33:H105)</f>
         <v>1.5</v>
       </c>
-      <c r="S14" s="27" t="s">
+      <c r="S14" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T14" s="9" t="s">
@@ -3711,20 +3723,20 @@
       </c>
       <c r="K15" s="15"/>
       <c r="L15" s="16"/>
-      <c r="O15" s="27">
+      <c r="O15" s="17">
         <v>13</v>
       </c>
-      <c r="P15" s="29" t="s">
+      <c r="P15" s="27" t="s">
         <v>210</v>
       </c>
-      <c r="Q15" s="31" t="s">
+      <c r="Q15" s="32" t="s">
         <v>232</v>
       </c>
-      <c r="R15" s="27">
+      <c r="R15" s="17">
         <f>SUMIF(C3:C105,Q15,H3:H105)</f>
         <v>0</v>
       </c>
-      <c r="S15" s="27" t="s">
+      <c r="S15" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T15" s="9" t="s">
@@ -3733,7 +3745,9 @@
     </row>
     <row r="16" spans="1:28" ht="40" customHeight="1">
       <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
+      <c r="B16" s="8" t="s">
+        <v>23</v>
+      </c>
       <c r="C16" s="16" t="s">
         <v>156</v>
       </c>
@@ -3758,20 +3772,20 @@
       </c>
       <c r="K16" s="15"/>
       <c r="L16" s="16"/>
-      <c r="O16" s="27">
+      <c r="O16" s="17">
         <v>14</v>
       </c>
-      <c r="P16" s="38" t="s">
+      <c r="P16" s="30" t="s">
         <v>250</v>
       </c>
-      <c r="Q16" s="37" t="s">
+      <c r="Q16" s="34" t="s">
         <v>182</v>
       </c>
-      <c r="R16" s="27">
+      <c r="R16" s="17">
         <f>SUMIF(C3:C105,Q16,H3:H105)</f>
         <v>3</v>
       </c>
-      <c r="S16" s="27" t="s">
+      <c r="S16" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T16" s="9" t="s">
@@ -3781,7 +3795,7 @@
     <row r="17" spans="1:20" ht="40" customHeight="1">
       <c r="A17" s="8"/>
       <c r="B17" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>164</v>
@@ -3807,20 +3821,20 @@
       </c>
       <c r="K17" s="15"/>
       <c r="L17" s="16"/>
-      <c r="O17" s="27">
+      <c r="O17" s="17">
         <v>15</v>
       </c>
-      <c r="P17" s="29" t="s">
+      <c r="P17" s="27" t="s">
         <v>211</v>
       </c>
-      <c r="Q17" s="31" t="s">
+      <c r="Q17" s="32" t="s">
         <v>233</v>
       </c>
-      <c r="R17" s="27">
+      <c r="R17" s="17">
         <f>SUMIF(C3:C105,Q17,H3:H105)</f>
         <v>3</v>
       </c>
-      <c r="S17" s="27" t="s">
+      <c r="S17" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T17" s="9" t="s">
@@ -3830,7 +3844,7 @@
     <row r="18" spans="1:20" ht="40" customHeight="1">
       <c r="A18" s="8"/>
       <c r="B18" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>151</v>
@@ -3855,20 +3869,20 @@
         <v>128</v>
       </c>
       <c r="M18" s="15"/>
-      <c r="O18" s="3">
+      <c r="O18" s="33">
         <v>16</v>
       </c>
-      <c r="P18" s="29" t="s">
+      <c r="P18" s="27" t="s">
         <v>212</v>
       </c>
-      <c r="Q18" s="31" t="s">
+      <c r="Q18" s="32" t="s">
         <v>234</v>
       </c>
-      <c r="R18" s="27">
+      <c r="R18" s="17">
         <f>SUMIF(C3:C105,Q18,H3:H105)</f>
         <v>4.5</v>
       </c>
-      <c r="S18" s="27" t="s">
+      <c r="S18" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T18" s="9" t="s">
@@ -3878,7 +3892,7 @@
     <row r="19" spans="1:20" ht="40" customHeight="1">
       <c r="A19" s="8"/>
       <c r="B19" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>130</v>
@@ -3905,20 +3919,20 @@
       <c r="K19" s="15"/>
       <c r="L19" s="15"/>
       <c r="M19" s="15"/>
-      <c r="O19" s="27">
+      <c r="O19" s="17">
         <v>17</v>
       </c>
-      <c r="P19" s="29" t="s">
+      <c r="P19" s="27" t="s">
         <v>213</v>
       </c>
-      <c r="Q19" s="31" t="s">
+      <c r="Q19" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="R19" s="27">
+      <c r="R19" s="17">
         <f>SUMIF(C3:C110,Q19,H3:H110)</f>
         <v>4.5</v>
       </c>
-      <c r="S19" s="27" t="s">
+      <c r="S19" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T19" s="9" t="s">
@@ -3928,7 +3942,7 @@
     <row r="20" spans="1:20" ht="40" customHeight="1">
       <c r="A20" s="8"/>
       <c r="B20" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C20" s="16" t="s">
         <v>161</v>
@@ -3955,20 +3969,20 @@
       <c r="K20" s="15"/>
       <c r="L20" s="15"/>
       <c r="M20" s="21"/>
-      <c r="O20" s="27">
+      <c r="O20" s="17">
         <v>18</v>
       </c>
-      <c r="P20" s="29" t="s">
+      <c r="P20" s="27" t="s">
         <v>214</v>
       </c>
-      <c r="Q20" s="37" t="s">
+      <c r="Q20" s="34" t="s">
         <v>236</v>
       </c>
-      <c r="R20" s="27">
+      <c r="R20" s="17">
         <f>SUMIF(C3:C110,Q20,H3:H110)</f>
         <v>1.5</v>
       </c>
-      <c r="S20" s="27" t="s">
+      <c r="S20" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T20" s="9" t="s">
@@ -3978,7 +3992,7 @@
     <row r="21" spans="1:20" ht="40" customHeight="1">
       <c r="A21" s="8"/>
       <c r="B21" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>152</v>
@@ -4005,20 +4019,20 @@
       <c r="K21" s="15"/>
       <c r="L21" s="15"/>
       <c r="M21" s="16"/>
-      <c r="O21" s="27">
+      <c r="O21" s="17">
         <v>19</v>
       </c>
-      <c r="P21" s="29" t="s">
+      <c r="P21" s="27" t="s">
         <v>215</v>
       </c>
-      <c r="Q21" s="31" t="s">
+      <c r="Q21" s="32" t="s">
         <v>237</v>
       </c>
-      <c r="R21" s="27">
+      <c r="R21" s="17">
         <f>SUMIF(C3:C110,Q21,H3:H110)</f>
         <v>3</v>
       </c>
-      <c r="S21" s="27" t="s">
+      <c r="S21" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T21" s="9" t="s">
@@ -4028,7 +4042,7 @@
     <row r="22" spans="1:20" ht="40" customHeight="1">
       <c r="A22" s="8"/>
       <c r="B22" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C22" s="16" t="s">
         <v>164</v>
@@ -4054,20 +4068,20 @@
       </c>
       <c r="K22" s="15"/>
       <c r="L22" s="16"/>
-      <c r="O22" s="27">
+      <c r="O22" s="17">
         <v>20</v>
       </c>
-      <c r="P22" s="28" t="s">
+      <c r="P22" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="Q22" s="31" t="s">
+      <c r="Q22" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="R22" s="27">
+      <c r="R22" s="17">
         <f>SUMIF(C3:C110,Q22,H3:H110)</f>
         <v>4.5</v>
       </c>
-      <c r="S22" s="27" t="s">
+      <c r="S22" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T22" s="9" t="s">
@@ -4077,7 +4091,7 @@
     <row r="23" spans="1:20" ht="40" customHeight="1">
       <c r="A23" s="8"/>
       <c r="B23" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>174</v>
@@ -4103,20 +4117,20 @@
       </c>
       <c r="K23" s="15"/>
       <c r="L23" s="16"/>
-      <c r="O23" s="27">
+      <c r="O23" s="17">
         <v>21</v>
       </c>
-      <c r="P23" s="29" t="s">
+      <c r="P23" s="27" t="s">
         <v>217</v>
       </c>
-      <c r="Q23" s="31" t="s">
+      <c r="Q23" s="32" t="s">
         <v>239</v>
       </c>
-      <c r="R23" s="27">
+      <c r="R23" s="17">
         <f>SUMIF(C3:C110,Q23,H3:H110)</f>
         <v>3</v>
       </c>
-      <c r="S23" s="27" t="s">
+      <c r="S23" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T23" s="9" t="s">
@@ -4126,7 +4140,7 @@
     <row r="24" spans="1:20" ht="40" customHeight="1">
       <c r="A24" s="8"/>
       <c r="B24" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>151</v>
@@ -4152,20 +4166,20 @@
       </c>
       <c r="K24" s="15"/>
       <c r="L24" s="16"/>
-      <c r="O24" s="27">
+      <c r="O24" s="17">
         <v>22</v>
       </c>
-      <c r="P24" s="29" t="s">
+      <c r="P24" s="27" t="s">
         <v>218</v>
       </c>
-      <c r="Q24" s="31" t="s">
+      <c r="Q24" s="32" t="s">
         <v>240</v>
       </c>
-      <c r="R24" s="27">
+      <c r="R24" s="17">
         <f>SUMIF(C3:C115,Q24,H3:H115)</f>
         <v>1.5</v>
       </c>
-      <c r="S24" s="27" t="s">
+      <c r="S24" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T24" s="9" t="s">
@@ -4175,7 +4189,7 @@
     <row r="25" spans="1:20" ht="40" customHeight="1">
       <c r="A25" s="8"/>
       <c r="B25" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>152</v>
@@ -4201,20 +4215,20 @@
       </c>
       <c r="K25" s="15"/>
       <c r="L25" s="16"/>
-      <c r="O25" s="27">
+      <c r="O25" s="17">
         <v>23</v>
       </c>
-      <c r="P25" s="29" t="s">
+      <c r="P25" s="27" t="s">
         <v>219</v>
       </c>
-      <c r="Q25" s="31" t="s">
+      <c r="Q25" s="32" t="s">
         <v>241</v>
       </c>
-      <c r="R25" s="27">
+      <c r="R25" s="17">
         <f>SUMIF(C3:C115,Q25,H3:H115)</f>
         <v>3</v>
       </c>
-      <c r="S25" s="27" t="s">
+      <c r="S25" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T25" s="9" t="s">
@@ -4224,7 +4238,7 @@
     <row r="26" spans="1:20" ht="40" customHeight="1">
       <c r="A26" s="8"/>
       <c r="B26" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>175</v>
@@ -4251,20 +4265,20 @@
       <c r="K26" s="15"/>
       <c r="L26" s="15"/>
       <c r="M26" s="16"/>
-      <c r="O26" s="27">
+      <c r="O26" s="17">
         <v>24</v>
       </c>
-      <c r="P26" s="29" t="s">
+      <c r="P26" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="Q26" s="31" t="s">
+      <c r="Q26" s="32" t="s">
         <v>242</v>
       </c>
-      <c r="R26" s="27">
+      <c r="R26" s="17">
         <f>SUMIF(C3:C115,Q26,H3:H115)</f>
         <v>4.5</v>
       </c>
-      <c r="S26" s="27" t="s">
+      <c r="S26" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T26" s="9" t="s">
@@ -4274,7 +4288,7 @@
     <row r="27" spans="1:20" ht="40" customHeight="1">
       <c r="A27" s="8"/>
       <c r="B27" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>129</v>
@@ -4301,20 +4315,20 @@
       <c r="K27" s="15"/>
       <c r="L27" s="6"/>
       <c r="M27" s="16"/>
-      <c r="O27" s="27">
+      <c r="O27" s="17">
         <v>25</v>
       </c>
-      <c r="P27" s="28" t="s">
+      <c r="P27" s="27" t="s">
         <v>221</v>
       </c>
-      <c r="Q27" s="31" t="s">
+      <c r="Q27" s="32" t="s">
         <v>243</v>
       </c>
-      <c r="R27" s="27">
+      <c r="R27" s="17">
         <f>SUMIF(C3:C115,Q27,H3:H115)</f>
         <v>6</v>
       </c>
-      <c r="S27" s="27" t="s">
+      <c r="S27" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T27" s="9" t="s">
@@ -4324,7 +4338,7 @@
     <row r="28" spans="1:20" ht="40" customHeight="1">
       <c r="A28" s="8"/>
       <c r="B28" s="8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C28" s="16" t="s">
         <v>130</v>
@@ -4350,20 +4364,20 @@
       </c>
       <c r="K28" s="15"/>
       <c r="L28" s="16"/>
-      <c r="O28" s="3">
+      <c r="O28" s="33">
         <v>26</v>
       </c>
-      <c r="P28" s="28" t="s">
+      <c r="P28" s="27" t="s">
         <v>222</v>
       </c>
-      <c r="Q28" s="31" t="s">
+      <c r="Q28" s="32" t="s">
         <v>244</v>
       </c>
-      <c r="R28" s="27">
+      <c r="R28" s="17">
         <f>SUMIF(C3:C115,Q28,H3:H115)</f>
         <v>1.5</v>
       </c>
-      <c r="S28" s="27" t="s">
+      <c r="S28" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T28" s="9" t="s">
@@ -4373,7 +4387,7 @@
     <row r="29" spans="1:20" ht="40" customHeight="1">
       <c r="A29" s="8"/>
       <c r="B29" s="8" t="s">
-        <v>36</v>
+        <v>258</v>
       </c>
       <c r="C29" s="16" t="s">
         <v>160</v>
@@ -4399,20 +4413,20 @@
       </c>
       <c r="K29" s="15"/>
       <c r="L29" s="16"/>
-      <c r="O29" s="27">
+      <c r="O29" s="17">
         <v>27</v>
       </c>
-      <c r="P29" s="28" t="s">
+      <c r="P29" s="27" t="s">
         <v>223</v>
       </c>
-      <c r="Q29" s="31" t="s">
+      <c r="Q29" s="32" t="s">
         <v>245</v>
       </c>
-      <c r="R29" s="27">
+      <c r="R29" s="17">
         <f>SUMIF(C3:C120,Q29,H3:H120)</f>
         <v>1.5</v>
       </c>
-      <c r="S29" s="27" t="s">
+      <c r="S29" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T29" s="9" t="s">
@@ -4448,20 +4462,20 @@
       </c>
       <c r="K30" s="15"/>
       <c r="L30" s="16"/>
-      <c r="O30" s="27">
+      <c r="O30" s="17">
         <v>28</v>
       </c>
-      <c r="P30" s="28" t="s">
+      <c r="P30" s="27" t="s">
         <v>224</v>
       </c>
-      <c r="Q30" s="31" t="s">
+      <c r="Q30" s="32" t="s">
         <v>246</v>
       </c>
-      <c r="R30" s="27">
+      <c r="R30" s="17">
         <f>SUMIF(C3:C120,Q30,H3:H120)</f>
         <v>3</v>
       </c>
-      <c r="S30" s="27" t="s">
+      <c r="S30" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T30" s="9" t="s">
@@ -4497,20 +4511,20 @@
       </c>
       <c r="K31" s="15"/>
       <c r="L31" s="16"/>
-      <c r="O31" s="27">
+      <c r="O31" s="17">
         <v>29</v>
       </c>
-      <c r="P31" s="36" t="s">
+      <c r="P31" s="29" t="s">
         <v>247</v>
       </c>
       <c r="Q31" s="35" t="s">
         <v>189</v>
       </c>
-      <c r="R31" s="27">
+      <c r="R31" s="17">
         <f>SUMIF(C3:C94,Q31,H3:H94)</f>
         <v>1.5</v>
       </c>
-      <c r="S31" s="27" t="s">
+      <c r="S31" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T31" s="9" t="s">
@@ -4546,20 +4560,20 @@
       </c>
       <c r="K32" s="15"/>
       <c r="L32" s="16"/>
-      <c r="O32" s="39">
+      <c r="O32" s="36">
         <v>30</v>
       </c>
-      <c r="P32" s="36" t="s">
+      <c r="P32" s="29" t="s">
         <v>153</v>
       </c>
       <c r="Q32" s="35" t="s">
         <v>149</v>
       </c>
-      <c r="R32" s="27">
+      <c r="R32" s="17">
         <f>SUMIF(C3:C94,Q32,H3:H94)</f>
         <v>4.5</v>
       </c>
-      <c r="S32" s="27" t="s">
+      <c r="S32" s="17" t="s">
         <v>251</v>
       </c>
       <c r="T32" s="9" t="s">
@@ -7039,443 +7053,443 @@
     <mergeCell ref="O1:T1"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
+  <conditionalFormatting sqref="C3">
+    <cfRule type="duplicateValues" dxfId="148" priority="154"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4">
+    <cfRule type="duplicateValues" dxfId="147" priority="153"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C5">
+    <cfRule type="duplicateValues" dxfId="146" priority="152"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C6">
+    <cfRule type="duplicateValues" dxfId="145" priority="60"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C7">
+    <cfRule type="duplicateValues" dxfId="144" priority="149"/>
+    <cfRule type="duplicateValues" dxfId="143" priority="150"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C8">
+    <cfRule type="duplicateValues" dxfId="142" priority="59"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9">
+    <cfRule type="duplicateValues" dxfId="141" priority="58"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C10">
+    <cfRule type="duplicateValues" dxfId="140" priority="146"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C11">
+    <cfRule type="duplicateValues" dxfId="139" priority="145"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C12">
+    <cfRule type="duplicateValues" dxfId="138" priority="57"/>
+    <cfRule type="duplicateValues" dxfId="137" priority="56"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C13">
+    <cfRule type="duplicateValues" dxfId="136" priority="142"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C14">
+    <cfRule type="duplicateValues" dxfId="135" priority="141"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C15:C16">
+    <cfRule type="duplicateValues" dxfId="134" priority="55"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C17">
+    <cfRule type="duplicateValues" dxfId="133" priority="54"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C18">
+    <cfRule type="duplicateValues" dxfId="132" priority="53"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C19">
+    <cfRule type="duplicateValues" dxfId="131" priority="137"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C20">
+    <cfRule type="duplicateValues" dxfId="130" priority="136"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C21">
+    <cfRule type="duplicateValues" dxfId="129" priority="135"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C22">
+    <cfRule type="duplicateValues" dxfId="128" priority="52"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C23">
+    <cfRule type="duplicateValues" dxfId="127" priority="133"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C24">
+    <cfRule type="duplicateValues" dxfId="126" priority="51"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C25">
+    <cfRule type="duplicateValues" dxfId="125" priority="50"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C26">
+    <cfRule type="duplicateValues" dxfId="124" priority="93"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C27">
+    <cfRule type="duplicateValues" dxfId="123" priority="49"/>
+    <cfRule type="duplicateValues" dxfId="122" priority="48"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C28">
+    <cfRule type="duplicateValues" dxfId="121" priority="47"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C29">
+    <cfRule type="duplicateValues" dxfId="120" priority="46"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C30">
+    <cfRule type="duplicateValues" dxfId="119" priority="45"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C31">
+    <cfRule type="duplicateValues" dxfId="118" priority="44"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C32">
+    <cfRule type="duplicateValues" dxfId="117" priority="42"/>
+    <cfRule type="duplicateValues" dxfId="116" priority="43"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C33">
+    <cfRule type="duplicateValues" dxfId="115" priority="115"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C34">
+    <cfRule type="duplicateValues" dxfId="114" priority="41"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C35">
+    <cfRule type="duplicateValues" dxfId="113" priority="37"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C36">
+    <cfRule type="duplicateValues" dxfId="112" priority="39"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C37:C38">
+    <cfRule type="duplicateValues" dxfId="111" priority="110"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C38:C39">
+    <cfRule type="duplicateValues" dxfId="110" priority="109"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C39:C40">
+    <cfRule type="duplicateValues" dxfId="109" priority="38"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C40:C41">
+    <cfRule type="duplicateValues" dxfId="108" priority="36"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C41:C42">
+    <cfRule type="duplicateValues" dxfId="107" priority="105"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C42:C43">
+    <cfRule type="duplicateValues" dxfId="106" priority="104"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C43:C44">
+    <cfRule type="duplicateValues" dxfId="105" priority="35"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C44:C45">
+    <cfRule type="duplicateValues" dxfId="104" priority="34"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C45:C46">
+    <cfRule type="duplicateValues" dxfId="103" priority="101"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C46:C47">
+    <cfRule type="duplicateValues" dxfId="102" priority="33"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C47:C48">
+    <cfRule type="duplicateValues" dxfId="101" priority="32"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C48:C49">
+    <cfRule type="duplicateValues" dxfId="100" priority="31"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C49:C50">
+    <cfRule type="duplicateValues" dxfId="99" priority="30"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C50:C51">
+    <cfRule type="duplicateValues" dxfId="98" priority="29"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C51:C52">
+    <cfRule type="duplicateValues" dxfId="97" priority="28"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C52:C53">
+    <cfRule type="duplicateValues" dxfId="96" priority="27"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C53:C54">
+    <cfRule type="duplicateValues" dxfId="95" priority="26"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C54:C55">
+    <cfRule type="duplicateValues" dxfId="94" priority="25"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C55:C56">
+    <cfRule type="duplicateValues" dxfId="93" priority="24"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C56:C57">
+    <cfRule type="duplicateValues" dxfId="92" priority="23"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C57:C58">
+    <cfRule type="duplicateValues" dxfId="91" priority="80"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C58:C59">
+    <cfRule type="duplicateValues" dxfId="90" priority="79"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C59:C60">
+    <cfRule type="duplicateValues" dxfId="89" priority="78"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C60:C61">
+    <cfRule type="duplicateValues" dxfId="88" priority="77"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C61:C62">
+    <cfRule type="duplicateValues" dxfId="87" priority="22"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C62:C63">
+    <cfRule type="duplicateValues" dxfId="86" priority="21"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C63:C64">
+    <cfRule type="duplicateValues" dxfId="85" priority="20"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C64:C65">
+    <cfRule type="duplicateValues" dxfId="84" priority="73"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C65:C66">
+    <cfRule type="duplicateValues" dxfId="83" priority="19"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C66:C67">
+    <cfRule type="duplicateValues" dxfId="82" priority="17"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C67:C68">
+    <cfRule type="duplicateValues" dxfId="81" priority="16"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C68:C69">
+    <cfRule type="duplicateValues" dxfId="80" priority="15"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C69">
-    <cfRule type="duplicateValues" dxfId="148" priority="68"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C3">
-    <cfRule type="duplicateValues" dxfId="147" priority="154"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C4">
-    <cfRule type="duplicateValues" dxfId="146" priority="153"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C5">
-    <cfRule type="duplicateValues" dxfId="145" priority="152"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C6">
-    <cfRule type="duplicateValues" dxfId="144" priority="60"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C7">
-    <cfRule type="duplicateValues" dxfId="143" priority="149"/>
-    <cfRule type="duplicateValues" dxfId="142" priority="150"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C8">
-    <cfRule type="duplicateValues" dxfId="141" priority="59"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C9">
-    <cfRule type="duplicateValues" dxfId="140" priority="58"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C10">
-    <cfRule type="duplicateValues" dxfId="139" priority="146"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C11">
-    <cfRule type="duplicateValues" dxfId="138" priority="145"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C12">
-    <cfRule type="duplicateValues" dxfId="137" priority="56"/>
-    <cfRule type="duplicateValues" dxfId="136" priority="57"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C13">
-    <cfRule type="duplicateValues" dxfId="135" priority="142"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C14">
-    <cfRule type="duplicateValues" dxfId="134" priority="141"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C15:C16">
-    <cfRule type="duplicateValues" dxfId="133" priority="55"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C17">
-    <cfRule type="duplicateValues" dxfId="132" priority="54"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C18">
-    <cfRule type="duplicateValues" dxfId="131" priority="53"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C19">
-    <cfRule type="duplicateValues" dxfId="130" priority="137"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C20">
-    <cfRule type="duplicateValues" dxfId="129" priority="136"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C21">
-    <cfRule type="duplicateValues" dxfId="128" priority="135"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C22">
-    <cfRule type="duplicateValues" dxfId="127" priority="52"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C23">
-    <cfRule type="duplicateValues" dxfId="126" priority="133"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C24">
-    <cfRule type="duplicateValues" dxfId="125" priority="51"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C25">
-    <cfRule type="duplicateValues" dxfId="124" priority="50"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C26">
-    <cfRule type="duplicateValues" dxfId="123" priority="93"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C27">
-    <cfRule type="duplicateValues" dxfId="122" priority="48"/>
-    <cfRule type="duplicateValues" dxfId="121" priority="49"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C28">
-    <cfRule type="duplicateValues" dxfId="120" priority="47"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C29">
-    <cfRule type="duplicateValues" dxfId="119" priority="46"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C30">
-    <cfRule type="duplicateValues" dxfId="118" priority="45"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C31">
-    <cfRule type="duplicateValues" dxfId="117" priority="44"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C32">
-    <cfRule type="duplicateValues" dxfId="116" priority="42"/>
-    <cfRule type="duplicateValues" dxfId="115" priority="43"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C33">
-    <cfRule type="duplicateValues" dxfId="114" priority="115"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C34">
-    <cfRule type="duplicateValues" dxfId="113" priority="41"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C35">
-    <cfRule type="duplicateValues" dxfId="112" priority="37"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C36">
-    <cfRule type="duplicateValues" dxfId="111" priority="39"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C37:C38">
-    <cfRule type="duplicateValues" dxfId="110" priority="110"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C38:C39">
-    <cfRule type="duplicateValues" dxfId="109" priority="109"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C39:C40">
-    <cfRule type="duplicateValues" dxfId="108" priority="38"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C40:C41">
-    <cfRule type="duplicateValues" dxfId="107" priority="36"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C41:C42">
-    <cfRule type="duplicateValues" dxfId="106" priority="105"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C42:C43">
-    <cfRule type="duplicateValues" dxfId="105" priority="104"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C43:C44">
-    <cfRule type="duplicateValues" dxfId="104" priority="35"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C44:C45">
-    <cfRule type="duplicateValues" dxfId="103" priority="34"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C45:C46">
-    <cfRule type="duplicateValues" dxfId="102" priority="101"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C46:C47">
-    <cfRule type="duplicateValues" dxfId="101" priority="33"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C47:C48">
-    <cfRule type="duplicateValues" dxfId="100" priority="32"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C48:C49">
-    <cfRule type="duplicateValues" dxfId="99" priority="31"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C49:C50">
-    <cfRule type="duplicateValues" dxfId="98" priority="30"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C50:C51">
-    <cfRule type="duplicateValues" dxfId="97" priority="29"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C51:C52">
-    <cfRule type="duplicateValues" dxfId="96" priority="28"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C52:C53">
-    <cfRule type="duplicateValues" dxfId="95" priority="27"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C53:C54">
-    <cfRule type="duplicateValues" dxfId="94" priority="26"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C54:C55">
-    <cfRule type="duplicateValues" dxfId="93" priority="25"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C55:C56">
-    <cfRule type="duplicateValues" dxfId="92" priority="24"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C56:C57">
-    <cfRule type="duplicateValues" dxfId="91" priority="23"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C57:C58">
-    <cfRule type="duplicateValues" dxfId="90" priority="80"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C58:C59">
-    <cfRule type="duplicateValues" dxfId="89" priority="79"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C59:C60">
-    <cfRule type="duplicateValues" dxfId="88" priority="78"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C60:C61">
-    <cfRule type="duplicateValues" dxfId="87" priority="77"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C61:C62">
-    <cfRule type="duplicateValues" dxfId="86" priority="22"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C62:C63">
-    <cfRule type="duplicateValues" dxfId="85" priority="21"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C63:C64">
-    <cfRule type="duplicateValues" dxfId="84" priority="20"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C64:C65">
-    <cfRule type="duplicateValues" dxfId="83" priority="73"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C65:C66">
-    <cfRule type="duplicateValues" dxfId="82" priority="19"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C66:C67">
-    <cfRule type="duplicateValues" dxfId="81" priority="17"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C67:C68">
-    <cfRule type="duplicateValues" dxfId="80" priority="16"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C68:C69">
-    <cfRule type="duplicateValues" dxfId="79" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="68"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C69:C70">
     <cfRule type="duplicateValues" dxfId="78" priority="67"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C70">
+    <cfRule type="duplicateValues" dxfId="77" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C70:C71">
-    <cfRule type="duplicateValues" dxfId="77" priority="66"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="66"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C71:C72">
-    <cfRule type="duplicateValues" dxfId="76" priority="65"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="65"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C72:C73">
-    <cfRule type="duplicateValues" dxfId="75" priority="64"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="64"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C73:C74">
-    <cfRule type="duplicateValues" dxfId="74" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C74:C75">
-    <cfRule type="duplicateValues" dxfId="73" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C75:C76">
-    <cfRule type="duplicateValues" dxfId="72" priority="11"/>
-    <cfRule type="duplicateValues" dxfId="71" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C76:C78">
-    <cfRule type="duplicateValues" dxfId="70" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C78:C80">
-    <cfRule type="duplicateValues" dxfId="69" priority="8"/>
     <cfRule type="duplicateValues" dxfId="68" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C79:C81">
-    <cfRule type="duplicateValues" dxfId="67" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C81:C83">
-    <cfRule type="duplicateValues" dxfId="66" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C82:C84">
-    <cfRule type="duplicateValues" dxfId="65" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C83:C85">
-    <cfRule type="duplicateValues" dxfId="64" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C86:C88">
-    <cfRule type="duplicateValues" dxfId="63" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C89:C91">
-    <cfRule type="duplicateValues" dxfId="62" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C99">
-    <cfRule type="duplicateValues" dxfId="61" priority="211"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="211"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C102">
-    <cfRule type="duplicateValues" dxfId="60" priority="210"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="210"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C103">
-    <cfRule type="duplicateValues" dxfId="59" priority="209"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="209"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C104">
-    <cfRule type="duplicateValues" dxfId="58" priority="208"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="208"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C106">
-    <cfRule type="duplicateValues" dxfId="57" priority="207"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="207"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C108">
-    <cfRule type="duplicateValues" dxfId="56" priority="206"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="206"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C111">
-    <cfRule type="duplicateValues" dxfId="55" priority="205"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="205"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C116">
-    <cfRule type="duplicateValues" dxfId="54" priority="204"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="204"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C118:C124">
-    <cfRule type="duplicateValues" dxfId="53" priority="203"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="203"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K7 N3:N13 L3:L6 L8:L13">
-    <cfRule type="duplicateValues" dxfId="52" priority="156"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="156"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L9">
-    <cfRule type="duplicateValues" dxfId="51" priority="198"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="198"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L15:L16">
-    <cfRule type="duplicateValues" dxfId="50" priority="123"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="123"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L17">
-    <cfRule type="duplicateValues" dxfId="49" priority="122"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="122"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L22">
-    <cfRule type="duplicateValues" dxfId="48" priority="199"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="199"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L23 L25">
-    <cfRule type="duplicateValues" dxfId="47" priority="200"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="200"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L30">
-    <cfRule type="duplicateValues" dxfId="46" priority="197"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="197"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L31">
-    <cfRule type="duplicateValues" dxfId="45" priority="196"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="196"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L34">
-    <cfRule type="duplicateValues" dxfId="44" priority="195"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="195"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L35">
-    <cfRule type="duplicateValues" dxfId="43" priority="194"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="194"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L36">
-    <cfRule type="duplicateValues" dxfId="42" priority="193"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="193"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L38">
-    <cfRule type="duplicateValues" dxfId="41" priority="192"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="192"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L39">
-    <cfRule type="duplicateValues" dxfId="40" priority="191"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="191"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L40">
-    <cfRule type="duplicateValues" dxfId="39" priority="190"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="190"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L42">
-    <cfRule type="duplicateValues" dxfId="38" priority="189"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="189"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L43">
-    <cfRule type="duplicateValues" dxfId="37" priority="188"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="188"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L44">
-    <cfRule type="duplicateValues" dxfId="36" priority="187"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="187"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L45">
-    <cfRule type="duplicateValues" dxfId="35" priority="186"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="186"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L47">
-    <cfRule type="duplicateValues" dxfId="34" priority="185"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="185"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L48">
-    <cfRule type="duplicateValues" dxfId="33" priority="184"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="184"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L50">
-    <cfRule type="duplicateValues" dxfId="32" priority="183"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="183"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L51">
-    <cfRule type="duplicateValues" dxfId="31" priority="182"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="182"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L52">
-    <cfRule type="duplicateValues" dxfId="30" priority="181"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="181"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L53">
-    <cfRule type="duplicateValues" dxfId="29" priority="180"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="180"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L56">
-    <cfRule type="duplicateValues" dxfId="28" priority="179"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="179"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L57">
-    <cfRule type="duplicateValues" dxfId="27" priority="178"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="178"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L58">
-    <cfRule type="duplicateValues" dxfId="26" priority="177"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="177"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L60">
-    <cfRule type="duplicateValues" dxfId="25" priority="176"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="176"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L62">
-    <cfRule type="duplicateValues" dxfId="24" priority="175"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="175"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L63">
-    <cfRule type="duplicateValues" dxfId="23" priority="174"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="174"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L66">
-    <cfRule type="duplicateValues" dxfId="22" priority="173"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="173"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L68">
-    <cfRule type="duplicateValues" dxfId="21" priority="172"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="172"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L69">
-    <cfRule type="duplicateValues" dxfId="20" priority="171"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="171"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L70">
-    <cfRule type="duplicateValues" dxfId="19" priority="170"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="170"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L74">
-    <cfRule type="duplicateValues" dxfId="18" priority="169"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="169"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L79">
-    <cfRule type="duplicateValues" dxfId="17" priority="168"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="168"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L80">
-    <cfRule type="duplicateValues" dxfId="16" priority="167"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="167"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L82">
-    <cfRule type="duplicateValues" dxfId="15" priority="166"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="166"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L86">
-    <cfRule type="duplicateValues" dxfId="14" priority="165"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="165"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L90">
-    <cfRule type="duplicateValues" dxfId="13" priority="164"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="164"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L98">
-    <cfRule type="duplicateValues" dxfId="12" priority="163"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="163"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L101">
-    <cfRule type="duplicateValues" dxfId="11" priority="162"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="162"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L102">
-    <cfRule type="duplicateValues" dxfId="10" priority="161"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="161"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L103">
-    <cfRule type="duplicateValues" dxfId="9" priority="160"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="160"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L105">
-    <cfRule type="duplicateValues" dxfId="8" priority="159"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="159"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L107">
-    <cfRule type="duplicateValues" dxfId="7" priority="158"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="158"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L110">
-    <cfRule type="duplicateValues" dxfId="6" priority="157"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="157"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L26:M26">
-    <cfRule type="duplicateValues" dxfId="5" priority="99"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="99"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="M21">
-    <cfRule type="duplicateValues" dxfId="4" priority="253"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="253"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="M26">
-    <cfRule type="duplicateValues" dxfId="3" priority="98"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="98"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="M27">
-    <cfRule type="duplicateValues" dxfId="2" priority="97"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="97"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="M11:N11">
-    <cfRule type="duplicateValues" dxfId="1" priority="257"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C70">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="257"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" scale="54" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
@@ -7487,6 +7501,7 @@
   <sheetData/>
   <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
</xml_diff>